<commit_message>
feat: agregue las hojas Casos y Explicacion al Excel
Agregue la hoja Casos con los 4 casos del enunciado (y una fila
"Caso propio" para completar con un sueldo real), cada fila con sus
propias formulas usando los rangos con nombre de Parametros, sin
depender de la hoja Boleta. Agregue la hoja Explicacion con cada
formula escrita en palabras, la formula en si y un ejemplo numerico
del Caso 1, pensada para alguien que no sabe contabilidad. Recalcule
con LibreOffice: 74 formulas en todo el libro, 0 errores, y los 4
casos coinciden al centavo con lo ya verificado en la app.
</commit_message>
<xml_diff>
--- a/SEMANA10/Sistema_De_Pago_Boleta/Excel/Boleta_de_pago.xlsx
+++ b/SEMANA10/Sistema_De_Pago_Boleta/Excel/Boleta_de_pago.xlsx
@@ -10,6 +10,8 @@
   <sheets>
     <sheet name="Parametros" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Boleta" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="Casos" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Explicacion" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName function="false" hidden="false" name="AFP_COMISION" vbProcedure="false">Parametros!$B$11</definedName>
@@ -32,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="108">
   <si>
     <t xml:space="preserve">PARAMETROS DEL CALCULO</t>
   </si>
@@ -170,6 +172,192 @@
   </si>
   <si>
     <t xml:space="preserve">Formulas vivas: cambia los datos de entrada y la boleta se recalcula sola.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Caso</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sueldo basico</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dias</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hijos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sistema</t>
+  </si>
+  <si>
+    <t xml:space="preserve">H.extra 25%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">H.extra 35%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Adelanto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sueldo comp.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Asig. familiar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">H.25% monto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">H.35% monto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total remun.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total desc.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EsSalud</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Caso 1 (con respuesta)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Caso 2 (con respuesta)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Si</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Caso 3 (con respuesta)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AFP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Caso 4 (evaluacion, sin respuesta)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Caso propio (completar con sueldo real)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Caso propio: reemplaza sueldo/dias/hijos/sistema con datos de una oferta laboral real (igual o mayor a la RMV). No uses datos personales reales.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EXPLICACION DE CADA FORMULA (para alguien que no sabe contabilidad)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Concepto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Que significa, en palabras</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Formula</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ejemplo numerico (Caso 1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Es cuanto del sueldo del mes le corresponde al trabajador segun los dias que realmente trabajo. Si trabajo el mes completo (30 dias), es el sueldo completo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sueldo basico / 30 x dias laborados</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2,500 / 30 x 30 dias = 2,500.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Un monto fijo que se le da al trabajador si tiene hijos, para ayudar con los gastos familiares. Es siempre el mismo monto, sin importar cuantos dias trabajo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10% de la RMV, si tiene hijos; si no, es 0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Caso 1 no tiene hijos -&gt; 0.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Horas extra 25% y 35%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lo que se paga por cada hora trabajada fuera del horario normal. Las primeras horas extra se pagan 25% mas caras que una hora normal, y las siguientes 35% mas caras.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(Sueldo basico / 30 / 8) x recargo x horas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Caso 1 no tiene horas extra -&gt; 0.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Es la suma de todo lo que el trabajador gana en el mes, antes de que le descuenten nada.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sueldo computable + asignacion familiar + horas extra 25% + horas extra 35%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2,500.00 + 0.00 + 0.00 + 0.00 = 2,500.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Es el dinero que se le descuenta al trabajador para su pension de jubilacion, si eligio el sistema publico (ONP) en vez de una AFP privada.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13% del total de remuneraciones (solo si eligio ONP)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2,500.00 x 13% = 325.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AFP (fondo, comision, seguro)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Si el trabajador eligio una AFP privada en vez de ONP, se le descuentan 3 montos distintos: uno va a su fondo de pension, otro es la comision que cobra la AFP por administrar ese fondo, y otro es un seguro.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cada uno es un % del total de remuneraciones (solo si eligio AFP)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Caso 1 eligio ONP -&gt; los 3 son 0.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Adelantos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dinero que la empresa ya le adelanto al trabajador durante el mes, y que por eso se le descuenta ahora de la boleta.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El monto que se ingreso, tal cual</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Caso 1 no tuvo adelantos -&gt; 0.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Es la suma de todo lo que se le resta al trabajador de su total de remuneraciones.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ONP (o AFP fondo+comision+seguro) + adelantos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">325.00 + 0.00 = 325.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Es el dinero que el trabajador realmente recibe en su cuenta o en efectivo: lo que gano, menos todo lo que se le descuenta.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total remuneraciones - total descuentos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2,500.00 - 325.00 = 2,175.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EsSalud (empleador)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Es un aporte para el seguro de salud del trabajador, pero NO se le descuenta a el: lo paga la empresa, por fuera de la boleta del trabajador.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9% del total de remuneraciones</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2,500.00 x 9% = 225.00</t>
   </si>
 </sst>
 </file>
@@ -335,65 +523,109 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="26">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -709,134 +941,134 @@
   <dimension ref="A1:C13"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="32"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="32"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="55"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="3" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="4" t="n">
+      <c r="B4" s="5" t="n">
         <v>1230</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="6" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="6" t="n">
+      <c r="B5" s="7" t="n">
         <v>0.1</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="6" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="6" t="n">
+      <c r="B6" s="7" t="n">
         <v>0.13</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C6" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="6" t="n">
+      <c r="B7" s="7" t="n">
         <v>0.09</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="C7" s="6" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B8" s="7" t="n">
+      <c r="B8" s="8" t="n">
         <v>1.25</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="C8" s="6" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B9" s="7" t="n">
+      <c r="B9" s="8" t="n">
         <v>1.35</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="C9" s="6" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B10" s="6" t="n">
+      <c r="B10" s="7" t="n">
         <v>0.1</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="C10" s="6" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3" t="s">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B11" s="6" t="n">
+      <c r="B11" s="7" t="n">
         <v>0.016</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="C11" s="6" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="3" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="6" t="n">
+      <c r="B12" s="7" t="n">
         <v>0.0135</v>
       </c>
-      <c r="C12" s="5" t="s">
+      <c r="C12" s="6" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="8" t="s">
+      <c r="A13" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="B13" s="8"/>
-      <c r="C13" s="8"/>
+      <c r="B13" s="9"/>
+      <c r="C13" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -861,234 +1093,234 @@
   <dimension ref="A1:C31"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="45"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="8" t="s">
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="B2" s="8"/>
-      <c r="C2" s="8"/>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="9" t="s">
+      <c r="B2" s="9"/>
+      <c r="C2" s="9"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="B4" s="9"/>
-      <c r="C4" s="9"/>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="s">
+      <c r="B4" s="10"/>
+      <c r="C4" s="10"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="B5" s="4" t="n">
+      <c r="B5" s="5" t="n">
         <v>2500</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="B6" s="10" t="n">
+      <c r="B6" s="11" t="n">
         <v>30</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B7" s="11" t="s">
+      <c r="B7" s="12" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="B8" s="11" t="s">
+      <c r="B8" s="12" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="B9" s="7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3" t="s">
+      <c r="B9" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="B10" s="7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3" t="s">
+      <c r="B10" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="B11" s="4" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="9" t="s">
+      <c r="B11" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="B13" s="9"/>
-      <c r="C13" s="9"/>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="3" t="s">
+      <c r="B13" s="10"/>
+      <c r="C13" s="10"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="B14" s="12" t="n">
+      <c r="B14" s="13" t="n">
         <f aca="false">ROUND(B5/30*B6,2)</f>
         <v>2500</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="3" t="s">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="B15" s="12" t="n">
+      <c r="B15" s="13" t="n">
         <f aca="false">ROUND(IF(B7="Si",RMV*PCT_ASIG_FAM,0),2)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="3" t="s">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="B16" s="12" t="n">
+      <c r="B16" s="13" t="n">
         <f aca="false">B5/30/8</f>
         <v>10.4166666666667</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="3" t="s">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="B17" s="12" t="n">
+      <c r="B17" s="13" t="n">
         <f aca="false">ROUND(B16*REC_25*B9,2)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="3" t="s">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="B18" s="12" t="n">
+      <c r="B18" s="13" t="n">
         <f aca="false">ROUND(B16*REC_35*B10,2)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="13" t="s">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="14" t="s">
         <v>36</v>
       </c>
-      <c r="B19" s="14" t="n">
+      <c r="B19" s="15" t="n">
         <f aca="false">B14+B15+B17+B18</f>
         <v>2500</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="3" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="B20" s="12" t="n">
+      <c r="B20" s="13" t="n">
         <f aca="false">IF(B8="ONP",ROUND(B19*PCT_ONP,2),0)</f>
         <v>325</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="3" t="s">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="B21" s="12" t="n">
+      <c r="B21" s="13" t="n">
         <f aca="false">IF(B8="AFP",ROUND(B19*AFP_FONDO,2),0)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="3" t="s">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="B22" s="12" t="n">
+      <c r="B22" s="13" t="n">
         <f aca="false">IF(B8="AFP",ROUND(B19*AFP_COMISION,2),0)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="3" t="s">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="B23" s="12" t="n">
+      <c r="B23" s="13" t="n">
         <f aca="false">IF(B8="AFP",ROUND(B19*AFP_SEGURO,2),0)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="3" t="s">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="B24" s="12" t="n">
+      <c r="B24" s="13" t="n">
         <f aca="false">B11</f>
         <v>0</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="3" t="s">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="B25" s="12" t="n">
+      <c r="B25" s="13" t="n">
         <f aca="false">B20+B21+B22+B23+B24</f>
         <v>325</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="13" t="s">
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="14" t="s">
         <v>42</v>
       </c>
-      <c r="B26" s="14" t="n">
+      <c r="B26" s="15" t="n">
         <f aca="false">B19-B25</f>
         <v>2175</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="9" t="s">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="B28" s="9"/>
-      <c r="C28" s="9"/>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="3" t="s">
+      <c r="B28" s="10"/>
+      <c r="C28" s="10"/>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="B29" s="12" t="n">
+      <c r="B29" s="13" t="n">
         <f aca="false">ROUND(B19*PCT_ESSALUD,2)</f>
         <v>225</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="8" t="s">
+      <c r="A31" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="B31" s="8"/>
-      <c r="C31" s="8"/>
+      <c r="B31" s="9"/>
+      <c r="C31" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -1117,4 +1349,714 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:T8"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="6" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="9" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="11" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="14" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="0" width="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="B1" s="16" t="s">
+        <v>47</v>
+      </c>
+      <c r="C1" s="16" t="s">
+        <v>48</v>
+      </c>
+      <c r="D1" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="E1" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="F1" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="G1" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="H1" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="I1" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="J1" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="K1" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="L1" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="M1" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N1" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="O1" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="P1" s="16" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q1" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="R1" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="S1" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="T1" s="16" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="17" t="s">
+        <v>61</v>
+      </c>
+      <c r="B2" s="18" t="n">
+        <v>2500</v>
+      </c>
+      <c r="C2" s="19" t="n">
+        <v>30</v>
+      </c>
+      <c r="D2" s="20" t="s">
+        <v>26</v>
+      </c>
+      <c r="E2" s="20" t="s">
+        <v>28</v>
+      </c>
+      <c r="F2" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" s="13" t="n">
+        <f aca="false">ROUND(B2/30*C2,2)</f>
+        <v>2500</v>
+      </c>
+      <c r="J2" s="13" t="n">
+        <f aca="false">ROUND(IF(D2="Si",RMV*PCT_ASIG_FAM,0),2)</f>
+        <v>0</v>
+      </c>
+      <c r="K2" s="13" t="n">
+        <f aca="false">ROUND((B2/30/8)*REC_25*F2,2)</f>
+        <v>0</v>
+      </c>
+      <c r="L2" s="13" t="n">
+        <f aca="false">ROUND((B2/30/8)*REC_35*G2,2)</f>
+        <v>0</v>
+      </c>
+      <c r="M2" s="15" t="n">
+        <f aca="false">I2+J2+K2+L2</f>
+        <v>2500</v>
+      </c>
+      <c r="N2" s="13" t="n">
+        <f aca="false">IF(E2="ONP",ROUND(M2*PCT_ONP,2),0)</f>
+        <v>325</v>
+      </c>
+      <c r="O2" s="13" t="n">
+        <f aca="false">IF(E2="AFP",ROUND(M2*AFP_FONDO,2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="P2" s="13" t="n">
+        <f aca="false">IF(E2="AFP",ROUND(M2*AFP_COMISION,2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="Q2" s="13" t="n">
+        <f aca="false">IF(E2="AFP",ROUND(M2*AFP_SEGURO,2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="R2" s="13" t="n">
+        <f aca="false">N2+O2+P2+Q2+H2</f>
+        <v>325</v>
+      </c>
+      <c r="S2" s="15" t="n">
+        <f aca="false">M2-R2</f>
+        <v>2175</v>
+      </c>
+      <c r="T2" s="13" t="n">
+        <f aca="false">ROUND(M2*PCT_ESSALUD,2)</f>
+        <v>225</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="17" t="s">
+        <v>62</v>
+      </c>
+      <c r="B3" s="18" t="n">
+        <v>1800</v>
+      </c>
+      <c r="C3" s="19" t="n">
+        <v>27</v>
+      </c>
+      <c r="D3" s="20" t="s">
+        <v>63</v>
+      </c>
+      <c r="E3" s="20" t="s">
+        <v>28</v>
+      </c>
+      <c r="F3" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" s="13" t="n">
+        <f aca="false">ROUND(B3/30*C3,2)</f>
+        <v>1620</v>
+      </c>
+      <c r="J3" s="13" t="n">
+        <f aca="false">ROUND(IF(D3="Si",RMV*PCT_ASIG_FAM,0),2)</f>
+        <v>123</v>
+      </c>
+      <c r="K3" s="13" t="n">
+        <f aca="false">ROUND((B3/30/8)*REC_25*F3,2)</f>
+        <v>0</v>
+      </c>
+      <c r="L3" s="13" t="n">
+        <f aca="false">ROUND((B3/30/8)*REC_35*G3,2)</f>
+        <v>0</v>
+      </c>
+      <c r="M3" s="15" t="n">
+        <f aca="false">I3+J3+K3+L3</f>
+        <v>1743</v>
+      </c>
+      <c r="N3" s="13" t="n">
+        <f aca="false">IF(E3="ONP",ROUND(M3*PCT_ONP,2),0)</f>
+        <v>226.59</v>
+      </c>
+      <c r="O3" s="13" t="n">
+        <f aca="false">IF(E3="AFP",ROUND(M3*AFP_FONDO,2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="P3" s="13" t="n">
+        <f aca="false">IF(E3="AFP",ROUND(M3*AFP_COMISION,2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="Q3" s="13" t="n">
+        <f aca="false">IF(E3="AFP",ROUND(M3*AFP_SEGURO,2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="R3" s="13" t="n">
+        <f aca="false">N3+O3+P3+Q3+H3</f>
+        <v>226.59</v>
+      </c>
+      <c r="S3" s="15" t="n">
+        <f aca="false">M3-R3</f>
+        <v>1516.41</v>
+      </c>
+      <c r="T3" s="13" t="n">
+        <f aca="false">ROUND(M3*PCT_ESSALUD,2)</f>
+        <v>156.87</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="17" t="s">
+        <v>64</v>
+      </c>
+      <c r="B4" s="18" t="n">
+        <v>3000</v>
+      </c>
+      <c r="C4" s="19" t="n">
+        <v>30</v>
+      </c>
+      <c r="D4" s="20" t="s">
+        <v>63</v>
+      </c>
+      <c r="E4" s="20" t="s">
+        <v>65</v>
+      </c>
+      <c r="F4" s="21" t="n">
+        <v>4</v>
+      </c>
+      <c r="G4" s="21" t="n">
+        <v>4</v>
+      </c>
+      <c r="H4" s="18" t="n">
+        <v>200</v>
+      </c>
+      <c r="I4" s="13" t="n">
+        <f aca="false">ROUND(B4/30*C4,2)</f>
+        <v>3000</v>
+      </c>
+      <c r="J4" s="13" t="n">
+        <f aca="false">ROUND(IF(D4="Si",RMV*PCT_ASIG_FAM,0),2)</f>
+        <v>123</v>
+      </c>
+      <c r="K4" s="13" t="n">
+        <f aca="false">ROUND((B4/30/8)*REC_25*F4,2)</f>
+        <v>62.5</v>
+      </c>
+      <c r="L4" s="13" t="n">
+        <f aca="false">ROUND((B4/30/8)*REC_35*G4,2)</f>
+        <v>67.5</v>
+      </c>
+      <c r="M4" s="15" t="n">
+        <f aca="false">I4+J4+K4+L4</f>
+        <v>3253</v>
+      </c>
+      <c r="N4" s="13" t="n">
+        <f aca="false">IF(E4="ONP",ROUND(M4*PCT_ONP,2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="O4" s="13" t="n">
+        <f aca="false">IF(E4="AFP",ROUND(M4*AFP_FONDO,2),0)</f>
+        <v>325.3</v>
+      </c>
+      <c r="P4" s="13" t="n">
+        <f aca="false">IF(E4="AFP",ROUND(M4*AFP_COMISION,2),0)</f>
+        <v>52.05</v>
+      </c>
+      <c r="Q4" s="13" t="n">
+        <f aca="false">IF(E4="AFP",ROUND(M4*AFP_SEGURO,2),0)</f>
+        <v>43.92</v>
+      </c>
+      <c r="R4" s="13" t="n">
+        <f aca="false">N4+O4+P4+Q4+H4</f>
+        <v>621.27</v>
+      </c>
+      <c r="S4" s="15" t="n">
+        <f aca="false">M4-R4</f>
+        <v>2631.73</v>
+      </c>
+      <c r="T4" s="13" t="n">
+        <f aca="false">ROUND(M4*PCT_ESSALUD,2)</f>
+        <v>292.77</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="17" t="s">
+        <v>66</v>
+      </c>
+      <c r="B5" s="18" t="n">
+        <v>4200</v>
+      </c>
+      <c r="C5" s="19" t="n">
+        <v>24</v>
+      </c>
+      <c r="D5" s="20" t="s">
+        <v>63</v>
+      </c>
+      <c r="E5" s="20" t="s">
+        <v>65</v>
+      </c>
+      <c r="F5" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="G5" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="H5" s="18" t="n">
+        <v>100</v>
+      </c>
+      <c r="I5" s="13" t="n">
+        <f aca="false">ROUND(B5/30*C5,2)</f>
+        <v>3360</v>
+      </c>
+      <c r="J5" s="13" t="n">
+        <f aca="false">ROUND(IF(D5="Si",RMV*PCT_ASIG_FAM,0),2)</f>
+        <v>123</v>
+      </c>
+      <c r="K5" s="13" t="n">
+        <f aca="false">ROUND((B5/30/8)*REC_25*F5,2)</f>
+        <v>43.75</v>
+      </c>
+      <c r="L5" s="13" t="n">
+        <f aca="false">ROUND((B5/30/8)*REC_35*G5,2)</f>
+        <v>47.25</v>
+      </c>
+      <c r="M5" s="15" t="n">
+        <f aca="false">I5+J5+K5+L5</f>
+        <v>3574</v>
+      </c>
+      <c r="N5" s="13" t="n">
+        <f aca="false">IF(E5="ONP",ROUND(M5*PCT_ONP,2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="O5" s="13" t="n">
+        <f aca="false">IF(E5="AFP",ROUND(M5*AFP_FONDO,2),0)</f>
+        <v>357.4</v>
+      </c>
+      <c r="P5" s="13" t="n">
+        <f aca="false">IF(E5="AFP",ROUND(M5*AFP_COMISION,2),0)</f>
+        <v>57.18</v>
+      </c>
+      <c r="Q5" s="13" t="n">
+        <f aca="false">IF(E5="AFP",ROUND(M5*AFP_SEGURO,2),0)</f>
+        <v>48.25</v>
+      </c>
+      <c r="R5" s="13" t="n">
+        <f aca="false">N5+O5+P5+Q5+H5</f>
+        <v>562.83</v>
+      </c>
+      <c r="S5" s="15" t="n">
+        <f aca="false">M5-R5</f>
+        <v>3011.17</v>
+      </c>
+      <c r="T5" s="13" t="n">
+        <f aca="false">ROUND(M5*PCT_ESSALUD,2)</f>
+        <v>321.66</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="17" t="s">
+        <v>67</v>
+      </c>
+      <c r="B6" s="18"/>
+      <c r="C6" s="19"/>
+      <c r="D6" s="20" t="s">
+        <v>26</v>
+      </c>
+      <c r="E6" s="20" t="s">
+        <v>28</v>
+      </c>
+      <c r="F6" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" s="13" t="n">
+        <f aca="false">ROUND(B6/30*C6,2)</f>
+        <v>0</v>
+      </c>
+      <c r="J6" s="13" t="n">
+        <f aca="false">ROUND(IF(D6="Si",RMV*PCT_ASIG_FAM,0),2)</f>
+        <v>0</v>
+      </c>
+      <c r="K6" s="13" t="n">
+        <f aca="false">ROUND((B6/30/8)*REC_25*F6,2)</f>
+        <v>0</v>
+      </c>
+      <c r="L6" s="13" t="n">
+        <f aca="false">ROUND((B6/30/8)*REC_35*G6,2)</f>
+        <v>0</v>
+      </c>
+      <c r="M6" s="15" t="n">
+        <f aca="false">I6+J6+K6+L6</f>
+        <v>0</v>
+      </c>
+      <c r="N6" s="13" t="n">
+        <f aca="false">IF(E6="ONP",ROUND(M6*PCT_ONP,2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="O6" s="13" t="n">
+        <f aca="false">IF(E6="AFP",ROUND(M6*AFP_FONDO,2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="P6" s="13" t="n">
+        <f aca="false">IF(E6="AFP",ROUND(M6*AFP_COMISION,2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="Q6" s="13" t="n">
+        <f aca="false">IF(E6="AFP",ROUND(M6*AFP_SEGURO,2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="R6" s="13" t="n">
+        <f aca="false">N6+O6+P6+Q6+H6</f>
+        <v>0</v>
+      </c>
+      <c r="S6" s="15" t="n">
+        <f aca="false">M6-R6</f>
+        <v>0</v>
+      </c>
+      <c r="T6" s="13" t="n">
+        <f aca="false">ROUND(M6*PCT_ESSALUD,2)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="22" t="s">
+        <v>68</v>
+      </c>
+      <c r="B8" s="22"/>
+      <c r="C8" s="22"/>
+      <c r="D8" s="22"/>
+      <c r="E8" s="22"/>
+      <c r="F8" s="22"/>
+      <c r="G8" s="22"/>
+      <c r="H8" s="22"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A8:H8"/>
+  </mergeCells>
+  <dataValidations count="10">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="D2" type="list">
+      <formula1>"No,Si"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E2" type="list">
+      <formula1>"ONP,AFP"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="D3" type="list">
+      <formula1>"No,Si"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E3" type="list">
+      <formula1>"ONP,AFP"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="D4" type="list">
+      <formula1>"No,Si"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E4" type="list">
+      <formula1>"ONP,AFP"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="D5" type="list">
+      <formula1>"No,Si"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E5" type="list">
+      <formula1>"ONP,AFP"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="D6" type="list">
+      <formula1>"No,Si"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E6" type="list">
+      <formula1>"ONP,AFP"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+  </dataValidations>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:D13"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="30"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="23" t="s">
+        <v>69</v>
+      </c>
+      <c r="B1" s="23"/>
+      <c r="C1" s="23"/>
+      <c r="D1" s="23"/>
+    </row>
+    <row r="3" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="16" t="s">
+        <v>70</v>
+      </c>
+      <c r="B3" s="16" t="s">
+        <v>71</v>
+      </c>
+      <c r="C3" s="16" t="s">
+        <v>72</v>
+      </c>
+      <c r="D3" s="16" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="24" t="s">
+        <v>33</v>
+      </c>
+      <c r="B4" s="25" t="s">
+        <v>74</v>
+      </c>
+      <c r="C4" s="25" t="s">
+        <v>75</v>
+      </c>
+      <c r="D4" s="25" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="24" t="s">
+        <v>34</v>
+      </c>
+      <c r="B5" s="25" t="s">
+        <v>77</v>
+      </c>
+      <c r="C5" s="25" t="s">
+        <v>78</v>
+      </c>
+      <c r="D5" s="25" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="24" t="s">
+        <v>80</v>
+      </c>
+      <c r="B6" s="25" t="s">
+        <v>81</v>
+      </c>
+      <c r="C6" s="25" t="s">
+        <v>82</v>
+      </c>
+      <c r="D6" s="25" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="24" t="s">
+        <v>36</v>
+      </c>
+      <c r="B7" s="25" t="s">
+        <v>84</v>
+      </c>
+      <c r="C7" s="25" t="s">
+        <v>85</v>
+      </c>
+      <c r="D7" s="25" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="24" t="s">
+        <v>28</v>
+      </c>
+      <c r="B8" s="25" t="s">
+        <v>87</v>
+      </c>
+      <c r="C8" s="25" t="s">
+        <v>88</v>
+      </c>
+      <c r="D8" s="25" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="24" t="s">
+        <v>90</v>
+      </c>
+      <c r="B9" s="25" t="s">
+        <v>91</v>
+      </c>
+      <c r="C9" s="25" t="s">
+        <v>92</v>
+      </c>
+      <c r="D9" s="25" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="24" t="s">
+        <v>94</v>
+      </c>
+      <c r="B10" s="25" t="s">
+        <v>95</v>
+      </c>
+      <c r="C10" s="25" t="s">
+        <v>96</v>
+      </c>
+      <c r="D10" s="25" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="24" t="s">
+        <v>41</v>
+      </c>
+      <c r="B11" s="25" t="s">
+        <v>98</v>
+      </c>
+      <c r="C11" s="25" t="s">
+        <v>99</v>
+      </c>
+      <c r="D11" s="25" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="24" t="s">
+        <v>42</v>
+      </c>
+      <c r="B12" s="25" t="s">
+        <v>101</v>
+      </c>
+      <c r="C12" s="25" t="s">
+        <v>102</v>
+      </c>
+      <c r="D12" s="25" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="24" t="s">
+        <v>104</v>
+      </c>
+      <c r="B13" s="25" t="s">
+        <v>105</v>
+      </c>
+      <c r="C13" s="25" t="s">
+        <v>106</v>
+      </c>
+      <c r="D13" s="25" t="s">
+        <v>107</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:D1"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: agregue el analisis y la tabla de fuentes dentro del Excel
Agregue a la hoja Explicacion las 4 preguntas ya respondidas (ONP vs
AFP, costo real para la empresa, dias laborados, horas extra) y la
pregunta 5 marcada como PENDIENTE hasta que tenga el sueldo de una
oferta laboral real. Tambien agregue la tabla de fuentes completa
(dato, valor, fuente, fecha de consulta), con la fila del caso
propio igual marcada PENDIENTE. Asi el Excel queda autocontenido,
sin depender del repositorio para ver el analisis. Recalcule con
LibreOffice: 74 formulas, 0 errores.
</commit_message>
<xml_diff>
--- a/SEMANA10/Sistema_De_Pago_Boleta/Excel/Boleta_de_pago.xlsx
+++ b/SEMANA10/Sistema_De_Pago_Boleta/Excel/Boleta_de_pago.xlsx
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="137">
   <si>
     <t xml:space="preserve">PARAMETROS DEL CALCULO</t>
   </si>
@@ -358,6 +358,93 @@
   </si>
   <si>
     <t xml:space="preserve">2,500.00 x 9% = 225.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ANALISIS - PREGUNTAS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. ONP o AFP (Caso 3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total remuneraciones: 3,253.00 (igual en ambos). Con ONP: 3,253.00 x 13% = 422.89 de descuento -&gt; neto 2,630.11. Con AFP Ejemplo: 325.30 + 52.05 + 43.92 = 421.27 -&gt; neto 2,631.73. La AFP deja S/ 1.62 mas este mes (12.95% vs 13%). No basta comparar los porcentajes porque no miden lo mismo: en AFP el 10% es ahorro propio del trabajador (rentabilidad variable), la comision y el seguro son gastos puros; en ONP el 13% no se ahorra, financia el sistema de reparto a cambio de una pension definida por ley. La diferencia de un mes no dice nada sobre el largo plazo (rentabilidad historica, anios para jubilarse, riesgo asumido).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2. Costo real para la empresa (Caso 3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Costo = Total remuneraciones + EsSalud = 3,253.00 + 292.77 = S/ 3,545.77. Del neto con AFP (2,631.73): 2,631.73 / 3,545.77 = 74.22% del costo del trabajador llega a el como neto. El 25.78% restante se reparte entre AFP, adelanto y EsSalud.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3. Dias laborados (Caso 2, 27 vs. 30 dias)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Con 27 dias: sueldo computable 1,620.00, total remuneraciones 1,743.00, ONP 226.59, neto 1,516.41 (caso original). Con 30 dias: sueldo computable 1,800.00, total remuneraciones 1,923.00, ONP 249.99, neto 1,673.01. Diferencia en el bruto (remuneraciones): 180.00. Diferencia en el neto: 156.60. El neto sube menos que el bruto porque esos 180 soles extra tambien pasan por el 13% de ONP: solo queda 87% (180.00 x 87% = 156.60, exacto). La asignacion familiar no cambia con los dias, asi que no afecta esta diferencia.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4. Horas extra (Caso 3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Horas extra 25% + 35% = 62.50 + 67.50 = 130.00. Total remuneraciones = 3,253.00. 130.00 / 3,253.00 = 4.00% del total de remuneraciones son horas extra.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5. Con datos reales</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PENDIENTE: falta el sueldo de una oferta laboral real (con el enlace y la fecha de consulta) para calcular el caso propio y el porcentaje del sueldo bruto que llega al trabajador, y compararlo con el de dos companeros.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TABLA DE FUENTES</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dato</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fecha de consulta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S/ 1,230.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dato del enunciado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10% de la RMV</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ley 25129</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ley 26790</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recargo horas extra</t>
+  </si>
+  <si>
+    <t xml:space="preserve">25% / 35%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AFP Ejemplo (fondo/comision/seguro)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.00% / 1.60% / 1.35%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Valores de prueba del enunciado; en datos reales usar la SBS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sueldo del caso propio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PENDIENTE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PENDIENTE (enlace de la oferta)</t>
   </si>
 </sst>
 </file>
@@ -523,7 +610,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="24">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -592,40 +679,32 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="167" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -1359,21 +1438,21 @@
   <dimension ref="A1:T8"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="6" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="9" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="11" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="14" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="6" style="1" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="9" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="11" style="1" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="14" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="1" width="10"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1438,29 +1517,29 @@
         <v>60</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="17" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="B2" s="18" t="n">
+      <c r="B2" s="17" t="n">
         <v>2500</v>
       </c>
-      <c r="C2" s="19" t="n">
+      <c r="C2" s="18" t="n">
         <v>30</v>
       </c>
-      <c r="D2" s="20" t="s">
+      <c r="D2" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="E2" s="20" t="s">
+      <c r="E2" s="19" t="s">
         <v>28</v>
       </c>
-      <c r="F2" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="G2" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="H2" s="18" t="n">
+      <c r="F2" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" s="17" t="n">
         <v>0</v>
       </c>
       <c r="I2" s="13" t="n">
@@ -1512,29 +1591,29 @@
         <v>225</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="17" t="s">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="B3" s="18" t="n">
+      <c r="B3" s="17" t="n">
         <v>1800</v>
       </c>
-      <c r="C3" s="19" t="n">
+      <c r="C3" s="18" t="n">
         <v>27</v>
       </c>
-      <c r="D3" s="20" t="s">
+      <c r="D3" s="19" t="s">
         <v>63</v>
       </c>
-      <c r="E3" s="20" t="s">
+      <c r="E3" s="19" t="s">
         <v>28</v>
       </c>
-      <c r="F3" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="G3" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="H3" s="18" t="n">
+      <c r="F3" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" s="17" t="n">
         <v>0</v>
       </c>
       <c r="I3" s="13" t="n">
@@ -1586,29 +1665,29 @@
         <v>156.87</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="17" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="B4" s="18" t="n">
+      <c r="B4" s="17" t="n">
         <v>3000</v>
       </c>
-      <c r="C4" s="19" t="n">
+      <c r="C4" s="18" t="n">
         <v>30</v>
       </c>
-      <c r="D4" s="20" t="s">
+      <c r="D4" s="19" t="s">
         <v>63</v>
       </c>
-      <c r="E4" s="20" t="s">
+      <c r="E4" s="19" t="s">
         <v>65</v>
       </c>
-      <c r="F4" s="21" t="n">
+      <c r="F4" s="20" t="n">
         <v>4</v>
       </c>
-      <c r="G4" s="21" t="n">
+      <c r="G4" s="20" t="n">
         <v>4</v>
       </c>
-      <c r="H4" s="18" t="n">
+      <c r="H4" s="17" t="n">
         <v>200</v>
       </c>
       <c r="I4" s="13" t="n">
@@ -1660,29 +1739,29 @@
         <v>292.77</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="17" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="B5" s="18" t="n">
+      <c r="B5" s="17" t="n">
         <v>4200</v>
       </c>
-      <c r="C5" s="19" t="n">
+      <c r="C5" s="18" t="n">
         <v>24</v>
       </c>
-      <c r="D5" s="20" t="s">
+      <c r="D5" s="19" t="s">
         <v>63</v>
       </c>
-      <c r="E5" s="20" t="s">
+      <c r="E5" s="19" t="s">
         <v>65</v>
       </c>
-      <c r="F5" s="21" t="n">
+      <c r="F5" s="20" t="n">
         <v>2</v>
       </c>
-      <c r="G5" s="21" t="n">
+      <c r="G5" s="20" t="n">
         <v>2</v>
       </c>
-      <c r="H5" s="18" t="n">
+      <c r="H5" s="17" t="n">
         <v>100</v>
       </c>
       <c r="I5" s="13" t="n">
@@ -1734,25 +1813,25 @@
         <v>321.66</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="17" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="B6" s="18"/>
-      <c r="C6" s="19"/>
-      <c r="D6" s="20" t="s">
+      <c r="B6" s="17"/>
+      <c r="C6" s="18"/>
+      <c r="D6" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="E6" s="20" t="s">
+      <c r="E6" s="19" t="s">
         <v>28</v>
       </c>
-      <c r="F6" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="G6" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="H6" s="18" t="n">
+      <c r="F6" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="17" t="n">
         <v>0</v>
       </c>
       <c r="I6" s="13" t="n">
@@ -1804,17 +1883,17 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="22" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="B8" s="22"/>
-      <c r="C8" s="22"/>
-      <c r="D8" s="22"/>
-      <c r="E8" s="22"/>
-      <c r="F8" s="22"/>
-      <c r="G8" s="22"/>
-      <c r="H8" s="22"/>
+      <c r="B8" s="9"/>
+      <c r="C8" s="9"/>
+      <c r="D8" s="9"/>
+      <c r="E8" s="9"/>
+      <c r="F8" s="9"/>
+      <c r="G8" s="9"/>
+      <c r="H8" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1877,21 +1956,21 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D37"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="55"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="1" width="30"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="23" t="s">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="B1" s="23"/>
-      <c r="C1" s="23"/>
-      <c r="D1" s="23"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
     </row>
     <row r="3" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="16" t="s">
@@ -1908,148 +1987,333 @@
       </c>
     </row>
     <row r="4" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="24" t="s">
+      <c r="A4" s="21" t="s">
         <v>33</v>
       </c>
-      <c r="B4" s="25" t="s">
+      <c r="B4" s="22" t="s">
         <v>74</v>
       </c>
-      <c r="C4" s="25" t="s">
+      <c r="C4" s="22" t="s">
         <v>75</v>
       </c>
-      <c r="D4" s="25" t="s">
+      <c r="D4" s="22" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="24" t="s">
+      <c r="A5" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="B5" s="25" t="s">
+      <c r="B5" s="22" t="s">
         <v>77</v>
       </c>
-      <c r="C5" s="25" t="s">
+      <c r="C5" s="22" t="s">
         <v>78</v>
       </c>
-      <c r="D5" s="25" t="s">
+      <c r="D5" s="22" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="24" t="s">
+      <c r="A6" s="21" t="s">
         <v>80</v>
       </c>
-      <c r="B6" s="25" t="s">
+      <c r="B6" s="22" t="s">
         <v>81</v>
       </c>
-      <c r="C6" s="25" t="s">
+      <c r="C6" s="22" t="s">
         <v>82</v>
       </c>
-      <c r="D6" s="25" t="s">
+      <c r="D6" s="22" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="24" t="s">
+      <c r="A7" s="21" t="s">
         <v>36</v>
       </c>
-      <c r="B7" s="25" t="s">
+      <c r="B7" s="22" t="s">
         <v>84</v>
       </c>
-      <c r="C7" s="25" t="s">
+      <c r="C7" s="22" t="s">
         <v>85</v>
       </c>
-      <c r="D7" s="25" t="s">
+      <c r="D7" s="22" t="s">
         <v>86</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="24" t="s">
+      <c r="A8" s="21" t="s">
         <v>28</v>
       </c>
-      <c r="B8" s="25" t="s">
+      <c r="B8" s="22" t="s">
         <v>87</v>
       </c>
-      <c r="C8" s="25" t="s">
+      <c r="C8" s="22" t="s">
         <v>88</v>
       </c>
-      <c r="D8" s="25" t="s">
+      <c r="D8" s="22" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="24" t="s">
+      <c r="A9" s="21" t="s">
         <v>90</v>
       </c>
-      <c r="B9" s="25" t="s">
+      <c r="B9" s="22" t="s">
         <v>91</v>
       </c>
-      <c r="C9" s="25" t="s">
+      <c r="C9" s="22" t="s">
         <v>92</v>
       </c>
-      <c r="D9" s="25" t="s">
+      <c r="D9" s="22" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="24" t="s">
+      <c r="A10" s="21" t="s">
         <v>94</v>
       </c>
-      <c r="B10" s="25" t="s">
+      <c r="B10" s="22" t="s">
         <v>95</v>
       </c>
-      <c r="C10" s="25" t="s">
+      <c r="C10" s="22" t="s">
         <v>96</v>
       </c>
-      <c r="D10" s="25" t="s">
+      <c r="D10" s="22" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="24" t="s">
+      <c r="A11" s="21" t="s">
         <v>41</v>
       </c>
-      <c r="B11" s="25" t="s">
+      <c r="B11" s="22" t="s">
         <v>98</v>
       </c>
-      <c r="C11" s="25" t="s">
+      <c r="C11" s="22" t="s">
         <v>99</v>
       </c>
-      <c r="D11" s="25" t="s">
+      <c r="D11" s="22" t="s">
         <v>100</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="24" t="s">
+      <c r="A12" s="21" t="s">
         <v>42</v>
       </c>
-      <c r="B12" s="25" t="s">
+      <c r="B12" s="22" t="s">
         <v>101</v>
       </c>
-      <c r="C12" s="25" t="s">
+      <c r="C12" s="22" t="s">
         <v>102</v>
       </c>
-      <c r="D12" s="25" t="s">
+      <c r="D12" s="22" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="24" t="s">
+      <c r="A13" s="21" t="s">
         <v>104</v>
       </c>
-      <c r="B13" s="25" t="s">
+      <c r="B13" s="22" t="s">
         <v>105</v>
       </c>
-      <c r="C13" s="25" t="s">
+      <c r="C13" s="22" t="s">
         <v>106</v>
       </c>
-      <c r="D13" s="25" t="s">
+      <c r="D13" s="22" t="s">
         <v>107</v>
       </c>
     </row>
+    <row r="16" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="23" t="s">
+        <v>108</v>
+      </c>
+      <c r="B16" s="23"/>
+      <c r="C16" s="23"/>
+      <c r="D16" s="23"/>
+    </row>
+    <row r="18" customFormat="false" ht="120" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="21" t="s">
+        <v>109</v>
+      </c>
+      <c r="B18" s="22" t="s">
+        <v>110</v>
+      </c>
+      <c r="C18" s="22"/>
+      <c r="D18" s="22"/>
+    </row>
+    <row r="20" customFormat="false" ht="120" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="21" t="s">
+        <v>111</v>
+      </c>
+      <c r="B20" s="22" t="s">
+        <v>112</v>
+      </c>
+      <c r="C20" s="22"/>
+      <c r="D20" s="22"/>
+    </row>
+    <row r="22" customFormat="false" ht="120" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="21" t="s">
+        <v>113</v>
+      </c>
+      <c r="B22" s="22" t="s">
+        <v>114</v>
+      </c>
+      <c r="C22" s="22"/>
+      <c r="D22" s="22"/>
+    </row>
+    <row r="24" customFormat="false" ht="120" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="21" t="s">
+        <v>115</v>
+      </c>
+      <c r="B24" s="22" t="s">
+        <v>116</v>
+      </c>
+      <c r="C24" s="22"/>
+      <c r="D24" s="22"/>
+    </row>
+    <row r="26" customFormat="false" ht="120" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="21" t="s">
+        <v>117</v>
+      </c>
+      <c r="B26" s="22" t="s">
+        <v>118</v>
+      </c>
+      <c r="C26" s="22"/>
+      <c r="D26" s="22"/>
+    </row>
+    <row r="28" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="23" t="s">
+        <v>119</v>
+      </c>
+      <c r="B28" s="23"/>
+      <c r="C28" s="23"/>
+      <c r="D28" s="23"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="16" t="s">
+        <v>120</v>
+      </c>
+      <c r="B30" s="16" t="s">
+        <v>2</v>
+      </c>
+      <c r="C30" s="16" t="s">
+        <v>3</v>
+      </c>
+      <c r="D30" s="16" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="22" t="s">
+        <v>4</v>
+      </c>
+      <c r="B31" s="22" t="s">
+        <v>122</v>
+      </c>
+      <c r="C31" s="22" t="s">
+        <v>5</v>
+      </c>
+      <c r="D31" s="22" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="22" t="s">
+        <v>34</v>
+      </c>
+      <c r="B32" s="22" t="s">
+        <v>124</v>
+      </c>
+      <c r="C32" s="22" t="s">
+        <v>125</v>
+      </c>
+      <c r="D32" s="22" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="22" t="s">
+        <v>28</v>
+      </c>
+      <c r="B33" s="22" t="s">
+        <v>126</v>
+      </c>
+      <c r="C33" s="22" t="s">
+        <v>9</v>
+      </c>
+      <c r="D33" s="22" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="22" t="s">
+        <v>60</v>
+      </c>
+      <c r="B34" s="22" t="s">
+        <v>127</v>
+      </c>
+      <c r="C34" s="22" t="s">
+        <v>128</v>
+      </c>
+      <c r="D34" s="22" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="22" t="s">
+        <v>129</v>
+      </c>
+      <c r="B35" s="22" t="s">
+        <v>130</v>
+      </c>
+      <c r="C35" s="22" t="s">
+        <v>13</v>
+      </c>
+      <c r="D35" s="22" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="22" t="s">
+        <v>131</v>
+      </c>
+      <c r="B36" s="22" t="s">
+        <v>132</v>
+      </c>
+      <c r="C36" s="22" t="s">
+        <v>133</v>
+      </c>
+      <c r="D36" s="22" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="22" t="s">
+        <v>134</v>
+      </c>
+      <c r="B37" s="22" t="s">
+        <v>135</v>
+      </c>
+      <c r="C37" s="22" t="s">
+        <v>136</v>
+      </c>
+      <c r="D37" s="22" t="s">
+        <v>135</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="8">
     <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A16:D16"/>
+    <mergeCell ref="B18:D18"/>
+    <mergeCell ref="B20:D20"/>
+    <mergeCell ref="B22:D22"/>
+    <mergeCell ref="B24:D24"/>
+    <mergeCell ref="B26:D26"/>
+    <mergeCell ref="A28:D28"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
feat: agregue que es cada concepto para presentar el trabajo
Agregue a la hoja Explicacion una tabla nueva, pensada para
presentarle el trabajo a alguien: por cada concepto (sueldo basico,
sueldo computable, asignacion familiar, horas extra, ONP, AFP
fondo/comision/seguro, adelantos, EsSalud y renta 5ta) explico de
donde sale o quien lo paga, para que sirve, y a que norma se debe.
Coloree cada fila: verde si es un ingreso (se suma), rojo si es un
descuento al trabajador, gris si es un aporte del empleador que no
afecta el neto, con su leyenda al final. Recalcule con LibreOffice:
74 formulas, 0 errores.
</commit_message>
<xml_diff>
--- a/SEMANA10/Sistema_De_Pago_Boleta/Excel/Boleta_de_pago.xlsx
+++ b/SEMANA10/Sistema_De_Pago_Boleta/Excel/Boleta_de_pago.xlsx
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="176">
   <si>
     <t xml:space="preserve">PARAMETROS DEL CALCULO</t>
   </si>
@@ -445,6 +445,123 @@
   </si>
   <si>
     <t xml:space="preserve">PENDIENTE (enlace de la oferta)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QUE ES CADA CONCEPTO (para presentar el trabajo)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">De donde sale / quien lo paga</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Para que sirve</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A que se debe (norma)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Es el punto de partida: lo que el trabajador y la empresa acordaron pagar por el mes completo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Es la base sobre la que se calculan todos los demas conceptos de la boleta.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Acuerdo laboral (contrato de trabajo)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Se ajusta del sueldo basico segun los dias realmente trabajados en el mes.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Paga al trabajador exactamente lo que le corresponde si no laboro el mes completo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D.S. 001-98-TR (formato de la boleta de pago)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No se descuenta: se SUMA al sueldo si el trabajador tiene hijos. Es un monto fijo (10% de la RMV).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ayuda economica para trabajadores con carga familiar.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Horas extra 25% / 35%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No se descuenta: se SUMA por cada hora trabajada fuera del horario normal.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Compensa el tiempo extra que el trabajador dedico a la empresa.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Se DESCUENTA al trabajador (13% del total de remuneraciones), si eligio el sistema publico de pensiones.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Financia el sistema de reparto: tu aporte no se ahorra a tu nombre, paga las pensiones actuales. A cambio, recibes una pension definida por ley al jubilarte.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AFP - Fondo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Se DESCUENTA al trabajador (10.00%), si eligio una AFP privada.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Es tu ahorro personal para la jubilacion; la AFP lo invierte y puede generar (o perder) rentabilidad.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sistema Privado de Pensiones (SPP)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AFP - Comision</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Se DESCUENTA al trabajador (1.60%), si eligio una AFP privada.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Es lo que cobra la AFP por administrar tu cuenta y tus inversiones. Es un gasto, no se recupera.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AFP - Seguro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Se DESCUENTA al trabajador (1.35%), si eligio una AFP privada.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cubre al trabajador y su familia en caso de invalidez o fallecimiento.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Se DESCUENTA al trabajador el monto que se ingreso, tal cual.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Es dinero que la empresa ya le entrego al trabajador durante el mes (un anticipo sobre su propio sueldo); por eso se resta ahora.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Acuerdo laboral</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NO se descuenta al trabajador: lo paga la EMPRESA, aparte de la boleta.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Financia el seguro de salud del trabajador (consultas, hospitalizacion, emergencias).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Renta de 5ta categoria (Nivel 3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Se DESCUENTA al trabajador solo si su sueldo anual proyectado supera las 7 UIT exoneradas.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Es el impuesto a la renta por trabajo dependiente; lo recauda el Estado a traves de SUNAT.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ley del Impuesto a la Renta (SUNAT)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verde = ingreso (se suma)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rojo = descuento (se resta al trabajador)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gris = aporte del empleador (no afecta el neto)</t>
   </si>
 </sst>
 </file>
@@ -458,7 +575,7 @@
     <numFmt numFmtId="167" formatCode="0.00"/>
     <numFmt numFmtId="168" formatCode="0"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="13">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -540,8 +657,14 @@
       <family val="0"/>
       <charset val="1"/>
     </font>
+    <font>
+      <sz val="9"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -557,7 +680,25 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFD9E1F2"/>
-        <bgColor rgb="FFCCFFFF"/>
+        <bgColor rgb="FFE2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE2EFDA"/>
+        <bgColor rgb="FFF2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFCE4E4"/>
+        <bgColor rgb="FFF2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor rgb="FFE2EFDA"/>
       </patternFill>
     </fill>
   </fills>
@@ -610,7 +751,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="33">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -704,6 +845,42 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -736,7 +913,7 @@
       <rgbColor rgb="FF808080"/>
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FFFFFFCC"/>
+      <rgbColor rgb="FFF2F2F2"/>
       <rgbColor rgb="FFCCFFFF"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
@@ -752,12 +929,12 @@
       <rgbColor rgb="FF0000FF"/>
       <rgbColor rgb="FF00CCFF"/>
       <rgbColor rgb="FFCCFFFF"/>
-      <rgbColor rgb="FFCCFFCC"/>
+      <rgbColor rgb="FFE2EFDA"/>
       <rgbColor rgb="FFFFFF99"/>
       <rgbColor rgb="FF99CCFF"/>
       <rgbColor rgb="FFFF99CC"/>
       <rgbColor rgb="FFCC99FF"/>
-      <rgbColor rgb="FFFFCC99"/>
+      <rgbColor rgb="FFFCE4E4"/>
       <rgbColor rgb="FF3366FF"/>
       <rgbColor rgb="FF33CCCC"/>
       <rgbColor rgb="FF99CC00"/>
@@ -1956,7 +2133,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D37"/>
+  <dimension ref="A1:D57"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="22"/>
@@ -2126,13 +2303,13 @@
         <v>107</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="23" t="s">
+    <row r="16" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="B16" s="23"/>
-      <c r="C16" s="23"/>
-      <c r="D16" s="23"/>
+      <c r="B16" s="2"/>
+      <c r="C16" s="2"/>
+      <c r="D16" s="2"/>
     </row>
     <row r="18" customFormat="false" ht="120" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="21" t="s">
@@ -2184,15 +2361,15 @@
       <c r="C26" s="22"/>
       <c r="D26" s="22"/>
     </row>
-    <row r="28" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="23" t="s">
+    <row r="28" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="B28" s="23"/>
-      <c r="C28" s="23"/>
-      <c r="D28" s="23"/>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B28" s="2"/>
+      <c r="C28" s="2"/>
+      <c r="D28" s="2"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="16" t="s">
         <v>120</v>
       </c>
@@ -2304,8 +2481,199 @@
         <v>135</v>
       </c>
     </row>
+    <row r="40" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="23" t="s">
+        <v>137</v>
+      </c>
+      <c r="B40" s="23"/>
+      <c r="C40" s="23"/>
+      <c r="D40" s="23"/>
+    </row>
+    <row r="42" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="16" t="s">
+        <v>70</v>
+      </c>
+      <c r="B42" s="16" t="s">
+        <v>138</v>
+      </c>
+      <c r="C42" s="16" t="s">
+        <v>139</v>
+      </c>
+      <c r="D42" s="16" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="24" t="s">
+        <v>47</v>
+      </c>
+      <c r="B43" s="25" t="s">
+        <v>141</v>
+      </c>
+      <c r="C43" s="25" t="s">
+        <v>142</v>
+      </c>
+      <c r="D43" s="25" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="24" t="s">
+        <v>33</v>
+      </c>
+      <c r="B44" s="25" t="s">
+        <v>144</v>
+      </c>
+      <c r="C44" s="25" t="s">
+        <v>145</v>
+      </c>
+      <c r="D44" s="25" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A45" s="24" t="s">
+        <v>34</v>
+      </c>
+      <c r="B45" s="25" t="s">
+        <v>147</v>
+      </c>
+      <c r="C45" s="25" t="s">
+        <v>148</v>
+      </c>
+      <c r="D45" s="25" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A46" s="24" t="s">
+        <v>149</v>
+      </c>
+      <c r="B46" s="25" t="s">
+        <v>150</v>
+      </c>
+      <c r="C46" s="25" t="s">
+        <v>151</v>
+      </c>
+      <c r="D46" s="25" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A47" s="26" t="s">
+        <v>28</v>
+      </c>
+      <c r="B47" s="27" t="s">
+        <v>152</v>
+      </c>
+      <c r="C47" s="27" t="s">
+        <v>153</v>
+      </c>
+      <c r="D47" s="27" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A48" s="26" t="s">
+        <v>154</v>
+      </c>
+      <c r="B48" s="27" t="s">
+        <v>155</v>
+      </c>
+      <c r="C48" s="27" t="s">
+        <v>156</v>
+      </c>
+      <c r="D48" s="27" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A49" s="26" t="s">
+        <v>158</v>
+      </c>
+      <c r="B49" s="27" t="s">
+        <v>159</v>
+      </c>
+      <c r="C49" s="27" t="s">
+        <v>160</v>
+      </c>
+      <c r="D49" s="27" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A50" s="26" t="s">
+        <v>161</v>
+      </c>
+      <c r="B50" s="27" t="s">
+        <v>162</v>
+      </c>
+      <c r="C50" s="27" t="s">
+        <v>163</v>
+      </c>
+      <c r="D50" s="27" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A51" s="26" t="s">
+        <v>94</v>
+      </c>
+      <c r="B51" s="27" t="s">
+        <v>164</v>
+      </c>
+      <c r="C51" s="27" t="s">
+        <v>165</v>
+      </c>
+      <c r="D51" s="27" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A52" s="28" t="s">
+        <v>44</v>
+      </c>
+      <c r="B52" s="29" t="s">
+        <v>167</v>
+      </c>
+      <c r="C52" s="29" t="s">
+        <v>168</v>
+      </c>
+      <c r="D52" s="29" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A53" s="26" t="s">
+        <v>169</v>
+      </c>
+      <c r="B53" s="27" t="s">
+        <v>170</v>
+      </c>
+      <c r="C53" s="27" t="s">
+        <v>171</v>
+      </c>
+      <c r="D53" s="27" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="30" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="31" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="32" t="s">
+        <v>175</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="9">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A16:D16"/>
     <mergeCell ref="B18:D18"/>
@@ -2314,6 +2682,7 @@
     <mergeCell ref="B24:D24"/>
     <mergeCell ref="B26:D26"/>
     <mergeCell ref="A28:D28"/>
+    <mergeCell ref="A40:D40"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>